<commit_message>
POCOR-6680: code enhance in students report cards | Status: Done
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/student_profile_template.xlsx
+++ b/webroot/export/customexcel/default_templates/student_profile_template.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="131">
   <si>
     <t>${Institutions.name}/${Institutions.code}</t>
   </si>
@@ -407,6 +407,18 @@
   </si>
   <si>
     <t>${"match": {"displayValue": "UserContacts.contact","rows": {"matchFrom": "UserContacts.id","matchTo": "UserContacts.id"}}}</t>
+  </si>
+  <si>
+    <t>Mother Name :</t>
+  </si>
+  <si>
+    <t>${StudentMoterDetails.mother_name}</t>
+  </si>
+  <si>
+    <t>Mother Contact :</t>
+  </si>
+  <si>
+    <t>${StudentMoterDetails.mother_contact}</t>
   </si>
 </sst>
 </file>
@@ -1325,8 +1337,24 @@
       <c r="E49" s="19"/>
     </row>
     <row r="50" spans="3:5" ht="12.75" customHeight="1"/>
-    <row r="51" spans="3:5" ht="12.75" customHeight="1"/>
-    <row r="52" spans="3:5" ht="12.75" customHeight="1"/>
+    <row r="51" spans="3:5" ht="12.75" customHeight="1">
+      <c r="C51" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D51" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="E51" s="20"/>
+    </row>
+    <row r="52" spans="3:5" ht="12.75" customHeight="1">
+      <c r="C52" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D52" s="20" t="s">
+        <v>130</v>
+      </c>
+      <c r="E52" s="20"/>
+    </row>
     <row r="53" spans="3:5" ht="12.75" customHeight="1"/>
     <row r="54" spans="3:5" ht="12.75" customHeight="1"/>
     <row r="55" spans="3:5" ht="12.75" customHeight="1"/>
@@ -2275,7 +2303,10 @@
     <row r="998" ht="12.75" customHeight="1"/>
     <row r="999" ht="12.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="28">
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
     <mergeCell ref="D34:E34"/>
     <mergeCell ref="D35:E35"/>
     <mergeCell ref="D36:E36"/>
@@ -2286,6 +2317,7 @@
     <mergeCell ref="D33:E33"/>
     <mergeCell ref="D28:E28"/>
     <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D51:E51"/>
     <mergeCell ref="D39:E39"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B3:F3"/>
@@ -2300,8 +2332,6 @@
     <mergeCell ref="D20:E20"/>
     <mergeCell ref="D21:E21"/>
     <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
POCOR-7316|Develop transcript and award placeholder|Status:Complete
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/student_profile_template.xlsx
+++ b/webroot/export/customexcel/default_templates/student_profile_template.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp2\htdocs\pocor-openemis-core\webroot\export\customexcel\default_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EABD84D-B1CB-4BE4-AF39-BF01D05D94B6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF9F3272-EA70-4E4F-B483-95834C3BD594}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="10" r:id="rId2"/>
+    <sheet name="Transcript" sheetId="10" r:id="rId2"/>
     <sheet name="Risks" sheetId="2" r:id="rId3"/>
     <sheet name="Classes" sheetId="3" r:id="rId4"/>
     <sheet name="Co-curricular" sheetId="4" r:id="rId5"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="152">
   <si>
     <t>${Institutions.name}/${Institutions.code}</t>
   </si>
@@ -432,18 +432,6 @@
     <t>Student Awards</t>
   </si>
   <si>
-    <t>${StudentAwards1.date}</t>
-  </si>
-  <si>
-    <t>${StudentAwards1.name}</t>
-  </si>
-  <si>
-    <t>${StudentAwards2.date}</t>
-  </si>
-  <si>
-    <t>${StudentAwards2.name}</t>
-  </si>
-  <si>
     <t>Academic Periods</t>
   </si>
   <si>
@@ -465,31 +453,37 @@
     <t>GPA</t>
   </si>
   <si>
-    <t xml:space="preserve">${Assessments.academic_period.name} </t>
-  </si>
-  <si>
-    <t>${EducationProgramme.Name}</t>
-  </si>
-  <si>
-    <t>${EducationGrade.Name}</t>
-  </si>
-  <si>
     <t>${"match": {"displayValue": "InstitutionSubjectStudentsWithName.name","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.id","matchTo": "InstitutionSubjectStudentsWithName.id"}}}</t>
   </si>
   <si>
     <t>${"match": {"displayValue": "InstitutionSubjectStudentsWithName.subjectName","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.id","matchTo": "InstitutionSubjectStudentsWithName.id"}}}</t>
   </si>
   <si>
-    <t>${"match": {"displayValue": "AssessmentItemResults.marks_formatted","type":"number","format":"2","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.education_subject_id","matchTo": "AssessmentItemResults.education_subject_id"},"columns": {"matchFrom": "AssessmentPeriods.id","matchTo": "AssessmentItemResults.assessment_period_id"}}}</t>
-  </si>
-  <si>
-    <t>${"match": {"displayValue": "InstitutionSubjectStudents.total_mark","type":"number","format":"2","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.education_subject_id","matchTo": "InstitutionSubjectStudentsWithName.education_subject_id"}}}</t>
-  </si>
-  <si>
     <t>{studentGPA}</t>
   </si>
   <si>
     <t>${Institutions.area}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "InstitutionSubjectStudentsWithName.academic_period_name","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.id","matchTo": "InstitutionSubjectStudentsWithName.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "InstitutionSubjectStudentsWithName.education_programme_name","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.id","matchTo": "InstitutionSubjectStudentsWithName.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "InstitutionSubjectStudentsWithName.education_grade_name","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.id","matchTo": "InstitutionSubjectStudentsWithName.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "InstitutionSubjectStudentsWithName.total_mark","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.id","matchTo": "InstitutionSubjectStudentsWithName.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "AssessmentItemResults.marks_formatted","type":"number","format":"2","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.id","matchTo": "AssessmentItemResults.id"},"columns": {"matchFrom": "AssessmentPeriods.id","matchTo": "AssessmentItemResults.assessment_period_id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "StudentAwards.date","rows": {"matchFrom": "StudentAwards.id","matchTo": "StudentAwards.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "StudentAwards.name","rows": {"matchFrom": "StudentAwards.id","matchTo": "StudentAwards.id"}}}</t>
   </si>
 </sst>
 </file>
@@ -591,7 +585,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -684,11 +678,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -742,7 +745,20 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -760,19 +776,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -785,6 +789,8 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1191,14 +1197,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:F1006"/>
+  <dimension ref="A1:F1006"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
     <col min="2" max="2" width="10.42578125" customWidth="1"/>
-    <col min="3" max="3" width="30.7109375" customWidth="1"/>
+    <col min="3" max="3" width="42.140625" customWidth="1"/>
     <col min="4" max="4" width="14.5703125" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="5" max="5" width="35.42578125" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="20.7109375" customWidth="1"/>
     <col min="8" max="27" width="15.5703125" customWidth="1"/>
@@ -1208,167 +1214,167 @@
   <sheetData>
     <row r="1" spans="2:6" ht="12.75" customHeight="1"/>
     <row r="2" spans="2:6" ht="12.75" customHeight="1">
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
     </row>
     <row r="3" spans="2:6" ht="12.75" customHeight="1">
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
     </row>
     <row r="4" spans="2:6" ht="12.75" customHeight="1">
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
     </row>
     <row r="6" spans="2:6" ht="12.75" customHeight="1">
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="39"/>
     </row>
     <row r="7" spans="2:6" ht="12.75" customHeight="1">
-      <c r="C7" s="34"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="34"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
     </row>
     <row r="8" spans="2:6" ht="12.75" customHeight="1">
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
     </row>
     <row r="9" spans="2:6" ht="12.75" customHeight="1">
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="39"/>
     </row>
     <row r="10" spans="2:6" ht="12.75" customHeight="1">
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
     </row>
     <row r="11" spans="2:6" ht="12.75" customHeight="1">
-      <c r="C11" s="34"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="34"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
     </row>
     <row r="12" spans="2:6" ht="12.75" customHeight="1">
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="39"/>
     </row>
     <row r="14" spans="2:6" ht="12.75" customHeight="1">
-      <c r="B14" s="31" t="s">
+      <c r="B14" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="31"/>
-      <c r="D14" s="31"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="31"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
     </row>
     <row r="15" spans="2:6" ht="12.75" customHeight="1">
       <c r="C15" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="D15" s="36" t="s">
+      <c r="D15" s="40" t="s">
         <v>119</v>
       </c>
-      <c r="E15" s="36"/>
+      <c r="E15" s="40"/>
     </row>
     <row r="16" spans="2:6" ht="12.75" customHeight="1">
       <c r="C16" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="D16" s="29" t="s">
+      <c r="D16" s="32" t="s">
         <v>121</v>
       </c>
-      <c r="E16" s="29"/>
+      <c r="E16" s="32"/>
     </row>
     <row r="17" spans="3:6" ht="12.75" customHeight="1">
       <c r="C17" s="20" t="s">
         <v>122</v>
       </c>
-      <c r="D17" s="29" t="s">
+      <c r="D17" s="32" t="s">
         <v>123</v>
       </c>
-      <c r="E17" s="29"/>
+      <c r="E17" s="32"/>
     </row>
     <row r="18" spans="3:6" ht="12.75" customHeight="1">
       <c r="C18" s="20" t="s">
         <v>124</v>
       </c>
-      <c r="D18" s="29" t="s">
+      <c r="D18" s="32" t="s">
         <v>125</v>
       </c>
-      <c r="E18" s="29"/>
+      <c r="E18" s="32"/>
     </row>
     <row r="19" spans="3:6" ht="12.75" customHeight="1">
       <c r="C19" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D19" s="35" t="s">
+      <c r="D19" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="E19" s="35"/>
+      <c r="E19" s="30"/>
     </row>
     <row r="20" spans="3:6" ht="12.75" customHeight="1">
       <c r="C20" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D20" s="35" t="s">
+      <c r="D20" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="E20" s="35"/>
+      <c r="E20" s="30"/>
     </row>
     <row r="21" spans="3:6" ht="12.75" customHeight="1">
       <c r="C21" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D21" s="35" t="s">
+      <c r="D21" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="E21" s="35"/>
+      <c r="E21" s="30"/>
     </row>
     <row r="22" spans="3:6" ht="12.75" customHeight="1">
       <c r="C22" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D22" s="35" t="s">
+      <c r="D22" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="E22" s="35"/>
+      <c r="E22" s="30"/>
     </row>
     <row r="23" spans="3:6" ht="12.75" customHeight="1">
       <c r="C23" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D23" s="35" t="s">
+      <c r="D23" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="E23" s="35"/>
+      <c r="E23" s="30"/>
     </row>
     <row r="24" spans="3:6" ht="12.75" customHeight="1">
       <c r="C24" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D24" s="35" t="s">
+      <c r="D24" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="E24" s="35"/>
+      <c r="E24" s="30"/>
     </row>
     <row r="25" spans="3:6" ht="12.75" customHeight="1">
       <c r="C25" t="s">
@@ -1383,204 +1389,201 @@
       <c r="C26" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D26" s="35" t="s">
+      <c r="D26" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="E26" s="35"/>
+      <c r="E26" s="30"/>
     </row>
     <row r="27" spans="3:6" ht="12.75" customHeight="1">
       <c r="C27" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D27" s="35" t="s">
+      <c r="D27" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="E27" s="35"/>
+      <c r="E27" s="30"/>
     </row>
     <row r="28" spans="3:6" ht="12.75" customHeight="1">
       <c r="C28" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D28" s="35" t="s">
+      <c r="D28" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="E28" s="35"/>
+      <c r="E28" s="30"/>
     </row>
     <row r="29" spans="3:6" ht="12.75" customHeight="1">
       <c r="C29" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D29" s="35" t="s">
+      <c r="D29" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="E29" s="35"/>
+      <c r="E29" s="30"/>
     </row>
     <row r="30" spans="3:6" ht="12.75" customHeight="1">
       <c r="C30" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D30" s="37" t="s">
+      <c r="D30" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="E30" s="37"/>
+      <c r="E30" s="31"/>
       <c r="F30" s="3"/>
     </row>
     <row r="31" spans="3:6" s="19" customFormat="1" ht="12.75" customHeight="1">
       <c r="C31" s="22"/>
-      <c r="D31" s="38"/>
-      <c r="E31" s="38"/>
+      <c r="D31" s="33"/>
+      <c r="E31" s="33"/>
       <c r="F31" s="3"/>
     </row>
     <row r="32" spans="3:6" s="19" customFormat="1" ht="12.75" customHeight="1">
       <c r="C32" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="D32" s="29" t="s">
+      <c r="D32" s="32" t="s">
         <v>127</v>
       </c>
-      <c r="E32" s="29"/>
+      <c r="E32" s="32"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="2:6" s="19" customFormat="1" ht="12.75" customHeight="1">
+    <row r="33" spans="1:6" s="19" customFormat="1" ht="12.75" customHeight="1">
       <c r="C33" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="D33" s="29" t="s">
+      <c r="D33" s="32" t="s">
         <v>129</v>
       </c>
-      <c r="E33" s="29"/>
+      <c r="E33" s="32"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="2:6" s="19" customFormat="1" ht="12.75" customHeight="1">
+    <row r="34" spans="1:6" s="19" customFormat="1" ht="12.75" customHeight="1">
       <c r="C34" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="D34" s="29" t="s">
+      <c r="D34" s="32" t="s">
         <v>131</v>
       </c>
-      <c r="E34" s="29"/>
+      <c r="E34" s="32"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="2:6" s="19" customFormat="1" ht="12.75" customHeight="1">
+    <row r="35" spans="1:6" s="19" customFormat="1" ht="12.75" customHeight="1">
       <c r="C35" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="D35" s="29" t="s">
-        <v>153</v>
+      <c r="D35" s="32" t="s">
+        <v>144</v>
       </c>
-      <c r="E35" s="29"/>
+      <c r="E35" s="32"/>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="2:6" s="19" customFormat="1" ht="12.75" customHeight="1">
+    <row r="36" spans="1:6" s="19" customFormat="1" ht="12.75" customHeight="1">
       <c r="C36"/>
-      <c r="D36" s="39"/>
-      <c r="E36" s="39"/>
+      <c r="D36" s="34"/>
+      <c r="E36" s="34"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="2:6" ht="15.75">
+    <row r="37" spans="1:6" ht="15.75">
       <c r="C37" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D37" s="35" t="s">
+      <c r="D37" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="E37" s="35"/>
-    </row>
-    <row r="38" spans="2:6" ht="12.75" customHeight="1">
+      <c r="E37" s="30"/>
+    </row>
+    <row r="38" spans="1:6" ht="12.75" customHeight="1">
       <c r="C38" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D38" s="35" t="s">
+      <c r="D38" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="E38" s="35"/>
-    </row>
-    <row r="39" spans="2:6" ht="12.75" customHeight="1">
+      <c r="E38" s="30"/>
+    </row>
+    <row r="39" spans="1:6" ht="12.75" customHeight="1">
       <c r="C39" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D39" s="35" t="s">
+      <c r="D39" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="E39" s="35"/>
-    </row>
-    <row r="40" spans="2:6" ht="12.75" customHeight="1">
+      <c r="E39" s="30"/>
+    </row>
+    <row r="40" spans="1:6" ht="12.75" customHeight="1">
       <c r="C40" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D40" s="35" t="s">
+      <c r="D40" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="E40" s="35"/>
-    </row>
-    <row r="41" spans="2:6" ht="12.75" customHeight="1">
+      <c r="E40" s="30"/>
+    </row>
+    <row r="41" spans="1:6" ht="12.75" customHeight="1">
       <c r="C41" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D41" s="35" t="s">
+      <c r="D41" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="E41" s="35"/>
-    </row>
-    <row r="42" spans="2:6" ht="12.75" customHeight="1">
+      <c r="E41" s="30"/>
+    </row>
+    <row r="42" spans="1:6" ht="12.75" customHeight="1">
       <c r="C42" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D42" s="35" t="s">
+      <c r="D42" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="E42" s="35"/>
-    </row>
-    <row r="43" spans="2:6" ht="12.75" customHeight="1">
+      <c r="E42" s="30"/>
+    </row>
+    <row r="43" spans="1:6" ht="12.75" customHeight="1">
       <c r="B43" s="23"/>
       <c r="C43" s="23"/>
       <c r="D43" s="23"/>
       <c r="E43" s="23"/>
       <c r="F43" s="23"/>
     </row>
-    <row r="44" spans="2:6">
+    <row r="44" spans="1:6">
       <c r="B44" s="25"/>
       <c r="C44" s="25"/>
       <c r="D44" s="25"/>
       <c r="E44" s="25"/>
       <c r="F44" s="25"/>
     </row>
-    <row r="45" spans="2:6" ht="12.75" customHeight="1">
-      <c r="B45" s="31" t="s">
+    <row r="45" spans="1:6" ht="12.75" customHeight="1">
+      <c r="B45" s="36" t="s">
         <v>133</v>
       </c>
-      <c r="C45" s="31"/>
-      <c r="D45" s="31"/>
-      <c r="E45" s="31"/>
-      <c r="F45" s="31"/>
-    </row>
-    <row r="46" spans="2:6" ht="12.75" customHeight="1">
+      <c r="C45" s="36"/>
+      <c r="D45" s="36"/>
+      <c r="E45" s="36"/>
+      <c r="F45" s="36"/>
+    </row>
+    <row r="46" spans="1:6" ht="12.75" customHeight="1">
       <c r="B46" s="25"/>
       <c r="C46" s="25"/>
       <c r="D46" s="25"/>
       <c r="E46" s="25"/>
       <c r="F46" s="25"/>
     </row>
-    <row r="47" spans="2:6" ht="12.75" customHeight="1">
-      <c r="B47" s="25"/>
-      <c r="C47" s="24" t="s">
-        <v>134</v>
+    <row r="47" spans="1:6" ht="12.75" customHeight="1">
+      <c r="A47" s="45"/>
+      <c r="B47" s="45"/>
+      <c r="C47" s="46" t="s">
+        <v>150</v>
       </c>
-      <c r="D47" s="29" t="s">
-        <v>135</v>
+      <c r="D47" s="32" t="s">
+        <v>151</v>
       </c>
-      <c r="E47" s="30"/>
+      <c r="E47" s="35"/>
       <c r="F47" s="25"/>
     </row>
-    <row r="48" spans="2:6" ht="12.75" customHeight="1">
+    <row r="48" spans="1:6" ht="12.75" customHeight="1">
       <c r="B48" s="25"/>
-      <c r="C48" s="24" t="s">
-        <v>136</v>
-      </c>
-      <c r="D48" s="29" t="s">
-        <v>137</v>
-      </c>
-      <c r="E48" s="30"/>
+      <c r="C48" s="24"/>
+      <c r="D48" s="32"/>
+      <c r="E48" s="35"/>
       <c r="F48" s="25"/>
     </row>
     <row r="49" ht="12.75" customHeight="1"/>
@@ -2543,25 +2546,6 @@
     <row r="1006" ht="12.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
     <mergeCell ref="D48:E48"/>
     <mergeCell ref="D47:E47"/>
     <mergeCell ref="B45:F45"/>
@@ -2578,6 +2562,25 @@
     <mergeCell ref="D16:E16"/>
     <mergeCell ref="D17:E17"/>
     <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D36:E36"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -2598,33 +2601,34 @@
     <col min="3" max="3" width="23.7109375" customWidth="1"/>
     <col min="4" max="4" width="19.5703125" customWidth="1"/>
     <col min="5" max="5" width="23.85546875" customWidth="1"/>
-    <col min="6" max="6" width="25.140625" customWidth="1"/>
+    <col min="6" max="6" width="35.7109375" customWidth="1"/>
+    <col min="7" max="7" width="37.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75">
       <c r="A1" s="26" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C1" s="26" t="s">
         <v>46</v>
       </c>
       <c r="D1" s="26" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="F1" s="26" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="G1" s="26" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="H1" s="26" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -2638,19 +2642,19 @@
         <v>147</v>
       </c>
       <c r="D2" s="27" t="s">
+        <v>141</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="F2" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="G2" s="27" t="s">
         <v>148</v>
       </c>
-      <c r="E2" s="27" t="s">
-        <v>149</v>
-      </c>
-      <c r="F2" s="27" t="s">
-        <v>150</v>
-      </c>
-      <c r="G2" s="27" t="s">
-        <v>151</v>
-      </c>
       <c r="H2" s="27" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="I2" s="28"/>
     </row>
@@ -2671,10 +2675,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15.75">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="40"/>
+      <c r="B1" s="41"/>
     </row>
     <row r="2" spans="1:3" ht="15.75">
       <c r="A2" s="6" t="s">
@@ -2727,14 +2731,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="12.75" customHeight="1">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
     </row>
     <row r="2" spans="1:7" ht="12.75" customHeight="1">
       <c r="A2" s="9" t="s">
@@ -4852,10 +4856,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="12.75" customHeight="1">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="41" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="40"/>
+      <c r="B1" s="41"/>
     </row>
     <row r="2" spans="1:3" ht="12.75" customHeight="1">
       <c r="A2" s="12" t="s">
@@ -4893,10 +4897,10 @@
       </c>
     </row>
     <row r="7" spans="1:3" ht="12.75" customHeight="1">
-      <c r="A7" s="40" t="s">
+      <c r="A7" s="41" t="s">
         <v>74</v>
       </c>
-      <c r="B7" s="40"/>
+      <c r="B7" s="41"/>
     </row>
     <row r="8" spans="1:3" ht="12.75" customHeight="1">
       <c r="A8" s="12" t="s">
@@ -5916,15 +5920,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="41" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="14"/>
@@ -33694,62 +33698,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="12.75" customHeight="1">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>92</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
     </row>
     <row r="2" spans="1:4" ht="12.75" customHeight="1">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="43" t="s">
         <v>93</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="43" t="s">
+      <c r="B2" s="43"/>
+      <c r="C2" s="44" t="s">
         <v>94</v>
       </c>
-      <c r="D2" s="43"/>
+      <c r="D2" s="44"/>
     </row>
     <row r="3" spans="1:4" ht="12.75" customHeight="1">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="43" t="s">
         <v>95</v>
       </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="43" t="s">
+      <c r="B3" s="43"/>
+      <c r="C3" s="44" t="s">
         <v>96</v>
       </c>
-      <c r="D3" s="43"/>
+      <c r="D3" s="44"/>
     </row>
     <row r="4" spans="1:4" ht="12.75" customHeight="1">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="43" t="s">
         <v>97</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="43" t="s">
+      <c r="B4" s="43"/>
+      <c r="C4" s="44" t="s">
         <v>98</v>
       </c>
-      <c r="D4" s="43"/>
+      <c r="D4" s="44"/>
     </row>
     <row r="5" spans="1:4" ht="12.75" customHeight="1">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="43" t="s">
         <v>99</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="43" t="s">
+      <c r="B5" s="43"/>
+      <c r="C5" s="44" t="s">
         <v>100</v>
       </c>
-      <c r="D5" s="43"/>
+      <c r="D5" s="44"/>
     </row>
     <row r="6" spans="1:4" ht="12.75" customHeight="1">
-      <c r="A6" s="42" t="s">
+      <c r="A6" s="43" t="s">
         <v>101</v>
       </c>
-      <c r="B6" s="42"/>
-      <c r="C6" s="43" t="s">
+      <c r="B6" s="43"/>
+      <c r="C6" s="44" t="s">
         <v>102</v>
       </c>
-      <c r="D6" s="43"/>
+      <c r="D6" s="44"/>
     </row>
     <row r="8" spans="1:4" ht="12.75" customHeight="1">
       <c r="A8" s="6" t="s">
@@ -34773,17 +34777,17 @@
     <row r="1001" ht="12.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:D3"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:D3"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -34809,12 +34813,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="12.75" customHeight="1">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
     </row>
     <row r="2" spans="1:5" ht="12.75" customHeight="1">
       <c r="A2" s="6" t="s">

</xml_diff>

<commit_message>
POCOR-7316|fixed inprogress and marks |Status:Complete
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/student_profile_template.xlsx
+++ b/webroot/export/customexcel/default_templates/student_profile_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp2\htdocs\pocor-openemis-core\webroot\export\customexcel\default_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF9F3272-EA70-4E4F-B483-95834C3BD594}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFF6EB40-29AF-4014-8FA6-862E09530782}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -585,7 +585,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -678,20 +678,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -736,9 +727,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -746,6 +734,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -759,9 +748,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -789,8 +775,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1197,7 +1184,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F1006"/>
+  <dimension ref="A1:F1005"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -1214,86 +1201,86 @@
   <sheetData>
     <row r="1" spans="2:6" ht="12.75" customHeight="1"/>
     <row r="2" spans="2:6" ht="12.75" customHeight="1">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
     </row>
     <row r="3" spans="2:6" ht="12.75" customHeight="1">
-      <c r="B3" s="38" t="s">
+      <c r="B3" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="38"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
     </row>
     <row r="4" spans="2:6" ht="12.75" customHeight="1">
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
     </row>
     <row r="6" spans="2:6" ht="12.75" customHeight="1">
-      <c r="C6" s="39" t="s">
+      <c r="C6" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="39"/>
-      <c r="E6" s="39"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
     </row>
     <row r="7" spans="2:6" ht="12.75" customHeight="1">
-      <c r="C7" s="39"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="39"/>
+      <c r="C7" s="38"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="38"/>
     </row>
     <row r="8" spans="2:6" ht="12.75" customHeight="1">
-      <c r="C8" s="39"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="39"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
     </row>
     <row r="9" spans="2:6" ht="12.75" customHeight="1">
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="39"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="38"/>
     </row>
     <row r="10" spans="2:6" ht="12.75" customHeight="1">
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="38"/>
     </row>
     <row r="11" spans="2:6" ht="12.75" customHeight="1">
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="39"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="38"/>
     </row>
     <row r="12" spans="2:6" ht="12.75" customHeight="1">
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="38"/>
     </row>
     <row r="14" spans="2:6" ht="12.75" customHeight="1">
-      <c r="B14" s="36" t="s">
+      <c r="B14" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="36"/>
-      <c r="F14" s="36"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
     </row>
     <row r="15" spans="2:6" ht="12.75" customHeight="1">
       <c r="C15" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="D15" s="40" t="s">
+      <c r="D15" s="39" t="s">
         <v>119</v>
       </c>
-      <c r="E15" s="40"/>
+      <c r="E15" s="39"/>
     </row>
     <row r="16" spans="2:6" ht="12.75" customHeight="1">
       <c r="C16" s="20" t="s">
@@ -1545,47 +1532,41 @@
       <c r="F43" s="23"/>
     </row>
     <row r="44" spans="1:6">
-      <c r="B44" s="25"/>
-      <c r="C44" s="25"/>
-      <c r="D44" s="25"/>
-      <c r="E44" s="25"/>
-      <c r="F44" s="25"/>
+      <c r="B44" s="24"/>
+      <c r="C44" s="24"/>
+      <c r="D44" s="24"/>
+      <c r="E44" s="24"/>
+      <c r="F44" s="24"/>
     </row>
     <row r="45" spans="1:6" ht="12.75" customHeight="1">
-      <c r="B45" s="36" t="s">
+      <c r="B45" s="35" t="s">
         <v>133</v>
       </c>
-      <c r="C45" s="36"/>
-      <c r="D45" s="36"/>
-      <c r="E45" s="36"/>
-      <c r="F45" s="36"/>
+      <c r="C45" s="35"/>
+      <c r="D45" s="35"/>
+      <c r="E45" s="35"/>
+      <c r="F45" s="35"/>
     </row>
     <row r="46" spans="1:6" ht="12.75" customHeight="1">
-      <c r="B46" s="25"/>
-      <c r="C46" s="25"/>
-      <c r="D46" s="25"/>
-      <c r="E46" s="25"/>
-      <c r="F46" s="25"/>
+      <c r="B46" s="24"/>
+      <c r="C46" s="24"/>
+      <c r="D46" s="24"/>
+      <c r="E46" s="24"/>
+      <c r="F46" s="24"/>
     </row>
     <row r="47" spans="1:6" ht="12.75" customHeight="1">
-      <c r="A47" s="45"/>
-      <c r="B47" s="45"/>
-      <c r="C47" s="46" t="s">
+      <c r="A47" s="29"/>
+      <c r="B47" s="29"/>
+      <c r="C47" s="29" t="s">
         <v>150</v>
       </c>
-      <c r="D47" s="32" t="s">
+      <c r="D47" s="44" t="s">
         <v>151</v>
       </c>
-      <c r="E47" s="35"/>
-      <c r="F47" s="25"/>
-    </row>
-    <row r="48" spans="1:6" ht="12.75" customHeight="1">
-      <c r="B48" s="25"/>
-      <c r="C48" s="24"/>
-      <c r="D48" s="32"/>
-      <c r="E48" s="35"/>
-      <c r="F48" s="25"/>
-    </row>
+      <c r="E47" s="44"/>
+      <c r="F47" s="24"/>
+    </row>
+    <row r="48" spans="1:6" ht="12.75" customHeight="1"/>
     <row r="49" ht="12.75" customHeight="1"/>
     <row r="50" ht="12.75" customHeight="1"/>
     <row r="51" ht="12.75" customHeight="1"/>
@@ -2543,10 +2524,8 @@
     <row r="1003" ht="12.75" customHeight="1"/>
     <row r="1004" ht="12.75" customHeight="1"/>
     <row r="1005" ht="12.75" customHeight="1"/>
-    <row r="1006" ht="12.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="35">
-    <mergeCell ref="D48:E48"/>
+  <mergeCells count="34">
     <mergeCell ref="D47:E47"/>
     <mergeCell ref="B45:F45"/>
     <mergeCell ref="B2:F2"/>
@@ -2606,57 +2585,57 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="25" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="25" t="s">
         <v>135</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="25" t="s">
         <v>136</v>
       </c>
-      <c r="E1" s="26" t="s">
+      <c r="E1" s="25" t="s">
         <v>137</v>
       </c>
-      <c r="F1" s="26" t="s">
+      <c r="F1" s="25" t="s">
         <v>138</v>
       </c>
-      <c r="G1" s="26" t="s">
+      <c r="G1" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="H1" s="26" t="s">
+      <c r="H1" s="25" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="26" t="s">
         <v>145</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="26" t="s">
         <v>146</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="26" t="s">
         <v>147</v>
       </c>
-      <c r="D2" s="27" t="s">
+      <c r="D2" s="26" t="s">
         <v>141</v>
       </c>
-      <c r="E2" s="27" t="s">
+      <c r="E2" s="26" t="s">
         <v>142</v>
       </c>
-      <c r="F2" s="29" t="s">
+      <c r="F2" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="G2" s="27" t="s">
+      <c r="G2" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="H2" s="27" t="s">
+      <c r="H2" s="26" t="s">
         <v>143</v>
       </c>
-      <c r="I2" s="28"/>
+      <c r="I2" s="27"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2675,10 +2654,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15.75">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="41"/>
+      <c r="B1" s="40"/>
     </row>
     <row r="2" spans="1:3" ht="15.75">
       <c r="A2" s="6" t="s">
@@ -2731,14 +2710,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="12.75" customHeight="1">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
     </row>
     <row r="2" spans="1:7" ht="12.75" customHeight="1">
       <c r="A2" s="9" t="s">
@@ -4856,10 +4835,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="12.75" customHeight="1">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="40" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="41"/>
+      <c r="B1" s="40"/>
     </row>
     <row r="2" spans="1:3" ht="12.75" customHeight="1">
       <c r="A2" s="12" t="s">
@@ -4897,10 +4876,10 @@
       </c>
     </row>
     <row r="7" spans="1:3" ht="12.75" customHeight="1">
-      <c r="A7" s="41" t="s">
+      <c r="A7" s="40" t="s">
         <v>74</v>
       </c>
-      <c r="B7" s="41"/>
+      <c r="B7" s="40"/>
     </row>
     <row r="8" spans="1:3" ht="12.75" customHeight="1">
       <c r="A8" s="12" t="s">
@@ -5920,15 +5899,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="14"/>
@@ -33698,62 +33677,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="12.75" customHeight="1">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="41" t="s">
         <v>92</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
     </row>
     <row r="2" spans="1:4" ht="12.75" customHeight="1">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="42" t="s">
         <v>93</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="44" t="s">
+      <c r="B2" s="42"/>
+      <c r="C2" s="43" t="s">
         <v>94</v>
       </c>
-      <c r="D2" s="44"/>
+      <c r="D2" s="43"/>
     </row>
     <row r="3" spans="1:4" ht="12.75" customHeight="1">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="42" t="s">
         <v>95</v>
       </c>
-      <c r="B3" s="43"/>
-      <c r="C3" s="44" t="s">
+      <c r="B3" s="42"/>
+      <c r="C3" s="43" t="s">
         <v>96</v>
       </c>
-      <c r="D3" s="44"/>
+      <c r="D3" s="43"/>
     </row>
     <row r="4" spans="1:4" ht="12.75" customHeight="1">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="42" t="s">
         <v>97</v>
       </c>
-      <c r="B4" s="43"/>
-      <c r="C4" s="44" t="s">
+      <c r="B4" s="42"/>
+      <c r="C4" s="43" t="s">
         <v>98</v>
       </c>
-      <c r="D4" s="44"/>
+      <c r="D4" s="43"/>
     </row>
     <row r="5" spans="1:4" ht="12.75" customHeight="1">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="42" t="s">
         <v>99</v>
       </c>
-      <c r="B5" s="43"/>
-      <c r="C5" s="44" t="s">
+      <c r="B5" s="42"/>
+      <c r="C5" s="43" t="s">
         <v>100</v>
       </c>
-      <c r="D5" s="44"/>
+      <c r="D5" s="43"/>
     </row>
     <row r="6" spans="1:4" ht="12.75" customHeight="1">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="42" t="s">
         <v>101</v>
       </c>
-      <c r="B6" s="43"/>
-      <c r="C6" s="44" t="s">
+      <c r="B6" s="42"/>
+      <c r="C6" s="43" t="s">
         <v>102</v>
       </c>
-      <c r="D6" s="44"/>
+      <c r="D6" s="43"/>
     </row>
     <row r="8" spans="1:4" ht="12.75" customHeight="1">
       <c r="A8" s="6" t="s">
@@ -34813,12 +34792,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="12.75" customHeight="1">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="41" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
     </row>
     <row r="2" spans="1:5" ht="12.75" customHeight="1">
       <c r="A2" s="6" t="s">

</xml_diff>

<commit_message>
Added GPA to excel file
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/student_profile_template.xlsx
+++ b/webroot/export/customexcel/default_templates/student_profile_template.xlsx
@@ -1,35 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\megha\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\pocor-openemis-core\webroot\export\customexcel\default_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{116EF0C7-E7B4-4018-AC10-48E6496F3615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A2AC4F-AF4F-4A74-B355-CB4945FD1A9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
     <sheet name="Risks" sheetId="2" r:id="rId2"/>
     <sheet name="Classes" sheetId="3" r:id="rId3"/>
-    <sheet name="Co-curricular" sheetId="4" r:id="rId4"/>
-    <sheet name="Learning Plan" sheetId="11" r:id="rId5"/>
-    <sheet name="Absences" sheetId="5" r:id="rId6"/>
-    <sheet name="Behaviours" sheetId="6" r:id="rId7"/>
-    <sheet name="Health Records" sheetId="7" r:id="rId8"/>
-    <sheet name="Counsellings" sheetId="8" r:id="rId9"/>
-    <sheet name="Cases" sheetId="9" r:id="rId10"/>
+    <sheet name="GPA" sheetId="13" r:id="rId4"/>
+    <sheet name="Co-curricular" sheetId="4" r:id="rId5"/>
+    <sheet name="Learning Plan" sheetId="11" r:id="rId6"/>
+    <sheet name="Absences" sheetId="5" r:id="rId7"/>
+    <sheet name="Behaviours" sheetId="6" r:id="rId8"/>
+    <sheet name="Health Records" sheetId="7" r:id="rId9"/>
+    <sheet name="Counsellings" sheetId="8" r:id="rId10"/>
+    <sheet name="Cases" sheetId="9" r:id="rId11"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="166">
   <si>
     <t>${Institutions.name}/${Institutions.code}</t>
   </si>
@@ -504,6 +505,30 @@
   <si>
     <t>${"match": {"displayValue": "InstitutionSubjectStudentsWithName.outcome_result","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.id","matchTo": "InstitutionSubjectStudentsWithName.id"}}}</t>
   </si>
+  <si>
+    <t>GPA</t>
+  </si>
+  <si>
+    <t>Cumulative GPA</t>
+  </si>
+  <si>
+    <t>GPA Start Date</t>
+  </si>
+  <si>
+    <t>GPA End Date</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "InstitutionStudentGradeGpa.gpa","rows": {"matchFrom": "InstitutionStudentGradeGpa.id","matchTo": "InstitutionStudentGradeGpa.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "InstitutionStudentGradeGpa.cumulative","rows": {"matchFrom": "InstitutionStudentGradeGpa.id","matchTo": "InstitutionStudentGradeGpa.id"}}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${"match": {"displayValue": "InstitutionStudentGradeGpa.start_date","rows": {"matchFrom": "InstitutionStudentGradeGpa.id","matchTo": "InstitutionStudentGradeGpa.id"}}} </t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "InstitutionStudentGradeGpa.end_date","rows": {"matchFrom": "InstitutionStudentGradeGpa.id","matchTo": "InstitutionStudentGradeGpa.id"}}}</t>
+  </si>
 </sst>
 </file>
 
@@ -676,7 +701,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -721,12 +746,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -739,16 +758,29 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1147,140 +1179,140 @@
   <sheetData>
     <row r="1" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
     </row>
     <row r="3" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="23"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
     </row>
     <row r="4" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
     </row>
     <row r="6" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
     </row>
     <row r="7" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
     </row>
     <row r="8" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="25"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
     </row>
     <row r="9" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
     </row>
     <row r="10" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="25"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
     </row>
     <row r="11" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
     </row>
     <row r="12" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
     </row>
     <row r="14" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
     </row>
     <row r="15" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C15" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D15" s="20" t="s">
+      <c r="D15" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="E15" s="20"/>
+      <c r="E15" s="24"/>
     </row>
     <row r="16" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C16" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D16" s="20" t="s">
+      <c r="D16" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="E16" s="20"/>
+      <c r="E16" s="24"/>
     </row>
     <row r="17" spans="3:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C17" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D17" s="20" t="s">
+      <c r="D17" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="E17" s="20"/>
+      <c r="E17" s="24"/>
     </row>
     <row r="18" spans="3:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C18" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="20" t="s">
+      <c r="D18" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="E18" s="20"/>
+      <c r="E18" s="24"/>
     </row>
     <row r="19" spans="3:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C19" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D19" s="20" t="s">
+      <c r="D19" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="E19" s="20"/>
+      <c r="E19" s="24"/>
     </row>
     <row r="20" spans="3:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C20" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D20" s="20" t="s">
+      <c r="D20" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="E20" s="20"/>
+      <c r="E20" s="24"/>
     </row>
     <row r="21" spans="3:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C21" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="20" t="s">
+      <c r="D21" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="E21" s="20"/>
+      <c r="E21" s="24"/>
     </row>
     <row r="22" spans="3:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C22" t="s">
@@ -1295,131 +1327,131 @@
       <c r="C23" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D23" s="20" t="s">
+      <c r="D23" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="E23" s="20"/>
+      <c r="E23" s="24"/>
     </row>
     <row r="24" spans="3:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C24" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D24" s="20" t="s">
+      <c r="D24" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="E24" s="20"/>
+      <c r="E24" s="24"/>
     </row>
     <row r="25" spans="3:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C25" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D25" s="20" t="s">
+      <c r="D25" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="E25" s="20"/>
+      <c r="E25" s="24"/>
     </row>
     <row r="26" spans="3:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C26" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D26" s="20" t="s">
+      <c r="D26" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="E26" s="20"/>
+      <c r="E26" s="24"/>
     </row>
     <row r="27" spans="3:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C27" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D27" s="21" t="s">
+      <c r="D27" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="E27" s="21"/>
+      <c r="E27" s="25"/>
       <c r="F27" s="7"/>
     </row>
     <row r="28" spans="3:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C28" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D28" s="21" t="s">
+      <c r="D28" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="E28" s="21"/>
+      <c r="E28" s="25"/>
       <c r="F28" s="7"/>
     </row>
     <row r="29" spans="3:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C29" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D29" s="21" t="s">
+      <c r="D29" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="E29" s="21"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="7"/>
     </row>
     <row r="31" spans="3:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C31" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D31" s="20" t="s">
+      <c r="D31" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="E31" s="20"/>
+      <c r="E31" s="24"/>
     </row>
     <row r="32" spans="3:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C32" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D32" s="20" t="s">
+      <c r="D32" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="E32" s="20"/>
+      <c r="E32" s="24"/>
     </row>
     <row r="33" spans="3:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C33" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D33" s="20" t="s">
+      <c r="D33" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="E33" s="20"/>
+      <c r="E33" s="24"/>
     </row>
     <row r="34" spans="3:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C34" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D34" s="20" t="s">
+      <c r="D34" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="E34" s="20"/>
+      <c r="E34" s="24"/>
     </row>
     <row r="35" spans="3:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C35" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="D35" s="20" t="s">
+      <c r="D35" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E35" s="20"/>
+      <c r="E35" s="24"/>
     </row>
     <row r="36" spans="3:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C36" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D36" s="20" t="s">
+      <c r="D36" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="E36" s="20"/>
+      <c r="E36" s="24"/>
     </row>
     <row r="38" spans="3:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="3:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C39" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="D39" s="20" t="s">
+      <c r="D39" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="E39" s="20"/>
+      <c r="E39" s="24"/>
     </row>
     <row r="40" spans="3:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="3:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1444,19 +1476,19 @@
       <c r="C51" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D51" s="20" t="s">
+      <c r="D51" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="E51" s="20"/>
+      <c r="E51" s="24"/>
     </row>
     <row r="52" spans="3:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C52" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D52" s="20" t="s">
+      <c r="D52" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="E52" s="20"/>
+      <c r="E52" s="24"/>
     </row>
     <row r="53" spans="3:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="54" spans="3:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2407,26 +2439,6 @@
     <row r="999" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="C6:E12"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D31:E31"/>
     <mergeCell ref="D39:E39"/>
     <mergeCell ref="D51:E51"/>
     <mergeCell ref="D52:E52"/>
@@ -2435,6 +2447,26 @@
     <mergeCell ref="D34:E34"/>
     <mergeCell ref="D35:E35"/>
     <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="C6:E12"/>
+    <mergeCell ref="B14:F14"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
@@ -2446,6 +2478,1068 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:E1000"/>
+  <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="72.88671875" customWidth="1"/>
+    <col min="2" max="2" width="51.6640625" customWidth="1"/>
+    <col min="3" max="4" width="41" customWidth="1"/>
+    <col min="5" max="7" width="22.5546875" customWidth="1"/>
+    <col min="8" max="27" width="15.5546875" customWidth="1"/>
+    <col min="28" max="256" width="19" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="27" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+    </row>
+    <row r="2" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="52" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="53" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="54" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="55" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="56" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="57" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="58" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="59" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="60" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="61" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="65" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="66" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="67" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="68" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="69" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="70" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="71" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="72" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="73" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="74" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="75" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="76" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="77" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="78" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="79" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="80" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="81" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="82" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="83" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="84" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="85" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="86" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="87" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="88" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="89" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="90" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="91" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="92" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="93" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="94" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="95" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="96" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="97" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="98" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="99" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="100" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="101" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="102" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="103" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="104" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="105" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="106" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="107" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="108" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="109" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="110" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="111" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="112" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="113" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="114" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="115" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="116" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="117" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="118" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="119" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="120" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="121" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="122" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="123" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="124" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="125" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="126" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="127" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="128" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="129" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="130" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="131" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="132" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="133" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="134" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="135" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="136" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="137" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="138" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="139" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="140" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="141" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="142" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="143" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="144" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="145" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="146" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="147" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="148" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="149" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="150" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="151" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="152" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="153" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="154" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="155" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="156" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="157" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="158" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="159" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="160" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="161" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="162" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="163" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="164" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="165" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="166" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="167" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="168" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="169" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="170" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="171" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="172" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="173" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="174" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="175" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="176" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="177" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="178" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="179" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="180" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="181" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="182" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="183" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="184" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="185" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="186" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="187" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="188" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="189" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="190" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="191" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="192" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="193" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="194" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="195" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="196" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="197" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="198" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="199" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="200" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="201" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="202" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="203" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="204" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="205" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="206" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="207" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="208" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="209" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="210" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="211" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="212" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="213" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="214" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="215" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="216" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="217" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="218" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="219" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="220" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="221" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="222" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="223" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="224" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="225" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="226" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="227" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="228" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="229" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="230" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="231" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="232" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="233" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="234" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="235" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="236" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="237" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="238" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="239" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="240" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="241" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="242" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="243" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="244" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="245" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="246" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="247" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="248" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="249" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="250" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="251" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="252" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="253" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="254" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="255" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="256" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="257" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="258" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="259" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="260" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="261" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="262" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="263" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="264" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="265" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="266" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="267" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="268" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="269" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="270" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="271" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="272" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="273" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="274" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="275" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="276" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="277" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="278" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="279" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="280" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="281" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="282" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="283" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="284" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="285" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="286" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="287" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="288" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="289" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="290" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="291" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="292" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="293" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="294" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="295" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="296" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="297" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="298" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="299" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="300" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="301" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="302" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="303" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="304" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="305" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="306" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="307" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="308" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="309" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="310" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="311" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="312" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="313" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="314" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="315" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="316" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="317" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="318" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="319" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="320" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="321" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="322" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="323" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="324" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="325" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="326" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="327" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="328" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="329" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="330" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="331" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="332" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="333" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="334" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="335" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="336" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="337" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="338" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="339" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="340" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="341" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="342" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="343" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="344" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="345" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="346" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="347" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="348" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="349" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="350" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="351" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="352" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="353" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="354" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="355" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="356" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="357" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="358" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="359" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="360" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="361" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="362" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="363" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="364" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="365" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="366" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="367" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="368" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="369" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="370" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="371" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="372" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="373" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="374" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="375" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="376" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="377" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="378" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="379" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="380" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="381" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="382" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="383" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="384" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="385" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="386" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="387" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="388" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="389" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="390" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="391" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="392" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="393" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="394" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="395" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="396" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="397" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="398" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="399" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="400" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="401" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="402" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="403" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="404" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="405" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="406" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="407" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="408" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="409" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="410" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="411" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="412" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="413" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="414" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="415" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="416" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="417" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="418" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="419" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="420" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="421" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="422" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="423" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="424" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="425" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="426" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="427" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="428" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="429" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="430" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="431" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="432" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="433" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="434" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="435" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="436" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="437" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="438" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="439" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="440" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="441" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="442" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="443" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="444" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="445" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="446" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="447" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="448" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="449" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="450" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="451" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="452" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="453" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="454" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="455" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="456" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="457" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="458" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="459" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="460" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="461" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="462" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="463" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="464" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="465" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="466" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="467" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="468" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="469" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="470" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="471" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="472" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="473" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="474" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="475" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="476" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="477" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="478" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="479" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="480" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="481" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="482" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="483" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="484" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="485" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="486" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="487" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="488" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="489" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="490" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="491" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="492" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="493" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="494" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="495" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="496" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="497" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="498" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="499" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="500" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="501" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="502" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="503" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="504" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="505" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="506" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="507" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="508" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="509" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="510" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="511" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="512" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="513" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="514" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="515" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="516" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="517" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="518" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="519" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="520" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="521" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="522" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="523" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="524" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="525" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="526" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="527" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="528" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="529" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="530" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="531" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="532" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="533" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="534" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="535" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="536" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="537" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="538" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="539" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="540" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="541" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="542" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="543" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="544" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="545" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="546" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="547" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="548" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="549" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="550" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="551" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="552" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="553" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="554" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="555" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="556" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="557" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="558" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="559" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="560" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="561" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="562" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="563" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="564" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="565" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="566" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="567" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="568" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="569" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="570" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="571" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="572" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="573" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="574" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="575" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="576" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="577" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="578" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="579" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="580" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="581" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="582" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="583" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="584" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="585" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="586" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="587" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="588" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="589" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="590" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="591" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="592" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="593" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="594" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="595" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="596" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="597" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="598" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="599" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="600" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="601" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="602" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="603" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="604" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="605" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="606" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="607" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="608" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="609" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="610" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="611" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="612" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="613" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="614" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="615" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="616" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="617" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="618" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="619" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="620" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="621" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="622" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="623" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="624" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="625" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="626" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="627" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="628" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="629" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="630" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="631" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="632" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="633" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="634" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="635" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="636" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="637" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="638" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="639" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="640" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="641" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="642" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="643" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="644" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="645" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="646" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="647" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="648" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="649" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="650" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="651" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="652" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="653" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="654" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="655" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="656" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="657" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="658" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="659" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="660" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="661" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="662" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="663" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="664" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="665" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="666" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="667" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="668" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="669" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="670" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="671" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="672" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="673" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="674" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="675" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="676" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="677" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="678" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="679" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="680" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="681" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="682" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="683" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="684" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="685" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="686" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="687" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="688" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="689" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="690" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="691" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="692" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="693" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="694" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="695" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="696" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="697" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="698" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="699" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="700" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="701" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="702" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="703" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="704" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="705" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="706" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="707" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="708" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="709" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="710" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="711" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="712" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="713" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="714" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="715" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="716" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="717" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="718" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="719" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="720" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="721" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="722" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="723" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="724" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="725" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="726" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="727" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="728" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="729" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="730" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="731" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="732" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="733" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="734" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="735" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="736" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="737" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="738" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="739" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="740" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="741" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="742" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="743" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="744" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="745" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="746" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="747" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="748" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="749" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="750" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="751" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="752" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="753" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="754" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="755" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="756" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="757" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="758" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="759" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="760" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="761" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="762" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="763" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="764" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="765" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="766" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="767" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="768" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="769" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="770" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="771" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="772" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="773" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="774" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="775" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="776" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="777" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="778" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="779" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="780" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="781" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="782" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="783" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="784" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="785" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="786" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="787" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="788" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="789" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="790" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="791" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="792" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="793" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="794" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="795" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="796" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="797" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="798" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="799" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="800" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="801" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="802" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="803" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="804" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="805" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="806" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="807" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="808" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="809" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="810" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="811" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="812" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="813" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="814" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="815" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="816" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="817" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="818" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="819" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="820" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="821" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="822" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="823" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="824" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="825" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="826" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="827" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="828" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="829" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="830" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="831" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="832" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="833" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="834" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="835" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="836" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="837" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="838" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="839" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="840" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="841" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="842" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="843" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="844" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="845" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="846" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="847" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="848" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="849" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="850" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="851" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="852" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="853" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="854" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="855" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="856" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="857" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="858" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="859" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="860" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="861" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="862" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="863" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="864" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="865" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="866" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="867" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="868" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="869" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="870" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="871" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="872" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="873" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="874" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="875" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="876" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="877" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="878" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="879" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="880" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="881" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="882" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="883" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="884" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="885" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="886" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="887" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="888" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="889" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="890" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="891" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="892" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="893" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="894" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="895" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="896" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="897" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="898" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="899" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="900" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="901" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="902" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="903" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="904" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="905" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="906" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="907" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="908" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="909" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="910" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="911" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="912" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="913" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="914" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="915" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="916" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="917" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="918" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="919" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="920" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="921" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="922" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="923" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="924" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="925" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="926" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="927" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="928" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="929" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="930" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="931" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="932" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="933" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="934" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="935" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="936" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="937" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="938" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="939" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="940" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="941" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="942" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="943" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="944" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="945" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="946" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="947" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="948" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="949" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="950" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="951" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="952" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="953" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="954" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="955" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="956" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="957" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="958" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="959" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="960" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="961" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="962" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="963" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="964" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="965" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="966" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="967" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="968" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="969" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="970" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="971" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="972" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="973" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="974" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="975" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="976" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="977" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="978" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="979" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="980" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="981" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="982" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="983" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="984" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="985" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="986" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="987" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="988" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="989" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="990" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="991" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="992" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="993" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="994" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="995" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="996" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="997" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="998" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="999" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1000" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
+  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;A</oddHeader>
+    <oddFooter>&amp;CPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:E1000"/>
   <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
@@ -2459,12 +3553,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="27" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
     </row>
     <row r="2" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
@@ -4628,6 +5722,58 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDC30773-BEC8-46B6-9100-E3B31A5AE447}">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.77734375" customWidth="1"/>
+    <col min="2" max="2" width="31.109375" customWidth="1"/>
+    <col min="3" max="3" width="27.6640625" customWidth="1"/>
+    <col min="4" max="4" width="31.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="31"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="31"/>
+    </row>
+    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.25">
+      <c r="A2" s="30" t="s">
+        <v>158</v>
+      </c>
+      <c r="B2" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>160</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="32" t="s">
+        <v>162</v>
+      </c>
+      <c r="B3" s="32" t="s">
+        <v>163</v>
+      </c>
+      <c r="C3" s="32" t="s">
+        <v>164</v>
+      </c>
+      <c r="D3" s="32" t="s">
+        <v>165</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:A1000"/>
   <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
@@ -5677,7 +6823,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AEB2BEF-5ABB-49D9-839F-8A25E0D64FDE}">
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
@@ -5760,7 +6906,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C989"/>
   <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
@@ -6822,7 +7968,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:Z990"/>
   <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
@@ -34598,7 +35744,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:D1001"/>
   <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
@@ -34613,62 +35759,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
     </row>
     <row r="2" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="28" t="s">
         <v>108</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="28" t="s">
+      <c r="B2" s="28"/>
+      <c r="C2" s="29" t="s">
         <v>109</v>
       </c>
-      <c r="D2" s="28"/>
+      <c r="D2" s="29"/>
     </row>
     <row r="3" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="28" t="s">
         <v>110</v>
       </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="28" t="s">
+      <c r="B3" s="28"/>
+      <c r="C3" s="29" t="s">
         <v>111</v>
       </c>
-      <c r="D3" s="28"/>
+      <c r="D3" s="29"/>
     </row>
     <row r="4" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="28" t="s">
         <v>112</v>
       </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="28" t="s">
+      <c r="B4" s="28"/>
+      <c r="C4" s="29" t="s">
         <v>113</v>
       </c>
-      <c r="D4" s="28"/>
+      <c r="D4" s="29"/>
     </row>
     <row r="5" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="28" t="s">
+      <c r="B5" s="28"/>
+      <c r="C5" s="29" t="s">
         <v>115</v>
       </c>
-      <c r="D5" s="28"/>
+      <c r="D5" s="29"/>
     </row>
     <row r="6" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="28" t="s">
         <v>116</v>
       </c>
-      <c r="B6" s="27"/>
-      <c r="C6" s="28" t="s">
+      <c r="B6" s="28"/>
+      <c r="C6" s="29" t="s">
         <v>117</v>
       </c>
-      <c r="D6" s="28"/>
+      <c r="D6" s="29"/>
     </row>
     <row r="8" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
@@ -35692,1079 +36838,17 @@
     <row r="1001" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:D3"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
-  </mergeCells>
-  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <headerFooter>
-    <oddHeader>&amp;C&amp;A</oddHeader>
-    <oddFooter>&amp;CPage &amp;P</oddFooter>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:E1000"/>
-  <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="72.88671875" customWidth="1"/>
-    <col min="2" max="2" width="51.6640625" customWidth="1"/>
-    <col min="3" max="4" width="41" customWidth="1"/>
-    <col min="5" max="7" width="22.5546875" customWidth="1"/>
-    <col min="8" max="27" width="15.5546875" customWidth="1"/>
-    <col min="28" max="256" width="19" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
-        <v>124</v>
-      </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-    </row>
-    <row r="2" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="53" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="55" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="67" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="68" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="69" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="70" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="71" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="72" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="73" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="74" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="75" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="76" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="77" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="78" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="79" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="80" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="81" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="82" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="83" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="84" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="85" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="86" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="87" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="88" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="89" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="90" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="91" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="92" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="93" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="94" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="95" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="96" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="97" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="98" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="99" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="100" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="101" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="102" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="103" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="104" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="105" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="106" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="107" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="108" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="109" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="110" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="111" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="112" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="113" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="114" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="115" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="116" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="117" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="118" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="119" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="120" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="121" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="122" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="123" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="124" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="125" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="126" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="127" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="128" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="129" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="130" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="131" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="132" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="133" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="134" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="135" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="136" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="137" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="138" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="139" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="140" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="141" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="142" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="143" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="144" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="145" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="146" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="147" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="148" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="149" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="150" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="151" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="152" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="153" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="154" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="155" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="156" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="157" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="158" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="159" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="160" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="161" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="162" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="163" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="164" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="165" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="166" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="167" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="168" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="169" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="170" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="171" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="172" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="173" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="174" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="175" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="176" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="177" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="178" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="179" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="180" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="181" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="182" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="183" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="184" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="185" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="186" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="187" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="188" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="189" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="190" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="191" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="192" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="193" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="194" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="195" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="196" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="197" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="198" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="199" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="200" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="201" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="202" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="203" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="204" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="205" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="206" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="207" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="208" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="209" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="210" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="211" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="212" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="213" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="214" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="215" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="216" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="217" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="218" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="219" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="220" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="221" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="222" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="223" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="224" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="225" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="226" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="227" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="228" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="229" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="230" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="231" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="232" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="233" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="234" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="235" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="236" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="237" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="238" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="239" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="240" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="241" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="242" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="243" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="244" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="245" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="246" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="247" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="248" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="249" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="250" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="251" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="252" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="253" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="254" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="255" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="256" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="257" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="258" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="259" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="260" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="261" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="262" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="263" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="264" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="265" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="266" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="267" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="268" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="269" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="270" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="271" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="272" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="273" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="274" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="275" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="276" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="277" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="278" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="279" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="280" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="281" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="282" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="283" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="284" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="285" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="286" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="287" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="288" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="289" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="290" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="291" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="292" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="293" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="294" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="295" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="296" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="297" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="298" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="299" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="300" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="301" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="302" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="303" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="304" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="305" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="306" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="307" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="308" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="309" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="310" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="311" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="312" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="313" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="314" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="315" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="316" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="317" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="318" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="319" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="320" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="321" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="322" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="323" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="324" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="325" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="326" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="327" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="328" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="329" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="330" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="331" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="332" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="333" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="334" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="335" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="336" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="337" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="338" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="339" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="340" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="341" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="342" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="343" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="344" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="345" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="346" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="347" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="348" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="349" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="350" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="351" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="352" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="353" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="354" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="355" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="356" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="357" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="358" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="359" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="360" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="361" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="362" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="363" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="364" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="365" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="366" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="367" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="368" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="369" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="370" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="371" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="372" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="373" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="374" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="375" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="376" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="377" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="378" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="379" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="380" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="381" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="382" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="383" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="384" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="385" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="386" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="387" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="388" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="389" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="390" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="391" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="392" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="393" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="394" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="395" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="396" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="397" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="398" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="399" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="400" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="401" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="402" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="403" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="404" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="405" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="406" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="407" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="408" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="409" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="410" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="411" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="412" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="413" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="414" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="415" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="416" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="417" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="418" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="419" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="420" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="421" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="422" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="423" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="424" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="425" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="426" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="427" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="428" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="429" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="430" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="431" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="432" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="433" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="434" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="435" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="436" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="437" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="438" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="439" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="440" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="441" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="442" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="443" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="444" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="445" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="446" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="447" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="448" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="449" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="450" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="451" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="452" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="453" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="454" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="455" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="456" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="457" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="458" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="459" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="460" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="461" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="462" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="463" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="464" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="465" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="466" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="467" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="468" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="469" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="470" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="471" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="472" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="473" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="474" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="475" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="476" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="477" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="478" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="479" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="480" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="481" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="482" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="483" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="484" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="485" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="486" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="487" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="488" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="489" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="490" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="491" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="492" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="493" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="494" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="495" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="496" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="497" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="498" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="499" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="500" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="501" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="502" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="503" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="504" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="505" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="506" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="507" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="508" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="509" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="510" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="511" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="512" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="513" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="514" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="515" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="516" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="517" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="518" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="519" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="520" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="521" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="522" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="523" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="524" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="525" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="526" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="527" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="528" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="529" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="530" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="531" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="532" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="533" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="534" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="535" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="536" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="537" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="538" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="539" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="540" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="541" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="542" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="543" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="544" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="545" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="546" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="547" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="548" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="549" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="550" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="551" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="552" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="553" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="554" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="555" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="556" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="557" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="558" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="559" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="560" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="561" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="562" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="563" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="564" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="565" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="566" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="567" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="568" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="569" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="570" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="571" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="572" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="573" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="574" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="575" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="576" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="577" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="578" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="579" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="580" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="581" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="582" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="583" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="584" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="585" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="586" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="587" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="588" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="589" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="590" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="591" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="592" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="593" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="594" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="595" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="596" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="597" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="598" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="599" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="600" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="601" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="602" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="603" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="604" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="605" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="606" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="607" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="608" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="609" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="610" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="611" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="612" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="613" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="614" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="615" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="616" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="617" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="618" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="619" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="620" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="621" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="622" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="623" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="624" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="625" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="626" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="627" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="628" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="629" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="630" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="631" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="632" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="633" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="634" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="635" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="636" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="637" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="638" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="639" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="640" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="641" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="642" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="643" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="644" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="645" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="646" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="647" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="648" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="649" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="650" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="651" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="652" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="653" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="654" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="655" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="656" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="657" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="658" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="659" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="660" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="661" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="662" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="663" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="664" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="665" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="666" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="667" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="668" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="669" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="670" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="671" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="672" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="673" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="674" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="675" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="676" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="677" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="678" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="679" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="680" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="681" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="682" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="683" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="684" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="685" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="686" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="687" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="688" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="689" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="690" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="691" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="692" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="693" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="694" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="695" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="696" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="697" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="698" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="699" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="700" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="701" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="702" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="703" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="704" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="705" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="706" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="707" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="708" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="709" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="710" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="711" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="712" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="713" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="714" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="715" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="716" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="717" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="718" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="719" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="720" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="721" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="722" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="723" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="724" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="725" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="726" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="727" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="728" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="729" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="730" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="731" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="732" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="733" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="734" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="735" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="736" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="737" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="738" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="739" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="740" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="741" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="742" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="743" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="744" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="745" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="746" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="747" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="748" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="749" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="750" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="751" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="752" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="753" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="754" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="755" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="756" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="757" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="758" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="759" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="760" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="761" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="762" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="763" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="764" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="765" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="766" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="767" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="768" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="769" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="770" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="771" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="772" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="773" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="774" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="775" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="776" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="777" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="778" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="779" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="780" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="781" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="782" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="783" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="784" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="785" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="786" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="787" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="788" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="789" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="790" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="791" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="792" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="793" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="794" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="795" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="796" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="797" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="798" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="799" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="800" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="801" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="802" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="803" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="804" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="805" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="806" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="807" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="808" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="809" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="810" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="811" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="812" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="813" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="814" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="815" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="816" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="817" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="818" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="819" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="820" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="821" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="822" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="823" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="824" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="825" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="826" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="827" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="828" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="829" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="830" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="831" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="832" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="833" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="834" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="835" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="836" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="837" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="838" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="839" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="840" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="841" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="842" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="843" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="844" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="845" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="846" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="847" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="848" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="849" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="850" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="851" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="852" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="853" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="854" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="855" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="856" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="857" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="858" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="859" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="860" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="861" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="862" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="863" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="864" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="865" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="866" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="867" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="868" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="869" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="870" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="871" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="872" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="873" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="874" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="875" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="876" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="877" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="878" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="879" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="880" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="881" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="882" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="883" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="884" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="885" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="886" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="887" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="888" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="889" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="890" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="891" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="892" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="893" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="894" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="895" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="896" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="897" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="898" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="899" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="900" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="901" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="902" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="903" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="904" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="905" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="906" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="907" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="908" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="909" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="910" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="911" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="912" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="913" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="914" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="915" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="916" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="917" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="918" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="919" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="920" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="921" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="922" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="923" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="924" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="925" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="926" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="927" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="928" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="929" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="930" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="931" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="932" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="933" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="934" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="935" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="936" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="937" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="938" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="939" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="940" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="941" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="942" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="943" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="944" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="945" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="946" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="947" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="948" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="949" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="950" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="951" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="952" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="953" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="954" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="955" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="956" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="957" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="958" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="959" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="960" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="961" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="962" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="963" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="964" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="965" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="966" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="967" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="968" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="969" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="970" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="971" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="972" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="973" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="974" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="975" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="976" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="977" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="978" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="979" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="980" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="981" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="982" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="983" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="984" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="985" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="986" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="987" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="988" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="989" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="990" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="991" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="992" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="993" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="994" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="995" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="996" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="997" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="998" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="999" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="1000" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-  </sheetData>
-  <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:D3"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
POCOR-8878||student report card placeholder
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/student_profile_template.xlsx
+++ b/webroot/export/customexcel/default_templates/student_profile_template.xlsx
@@ -5,39 +5,40 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\pocor-openemis-core\webroot\export\customexcel\default_templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6470" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6470" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
     <sheet name="Programmes" sheetId="2" r:id="rId2"/>
     <sheet name="Competencies" sheetId="3" r:id="rId3"/>
-    <sheet name="Assessments" sheetId="4" r:id="rId4"/>
-    <sheet name="Risks" sheetId="5" r:id="rId5"/>
-    <sheet name="Classes" sheetId="6" r:id="rId6"/>
-    <sheet name="GPA" sheetId="7" r:id="rId7"/>
-    <sheet name="Co-curricular" sheetId="8" r:id="rId8"/>
-    <sheet name="Learning Plan" sheetId="9" r:id="rId9"/>
-    <sheet name="Absences" sheetId="10" r:id="rId10"/>
-    <sheet name="Behaviours" sheetId="11" r:id="rId11"/>
-    <sheet name="Health Records" sheetId="12" r:id="rId12"/>
-    <sheet name="Counsellings" sheetId="13" r:id="rId13"/>
-    <sheet name="Cases" sheetId="14" r:id="rId14"/>
+    <sheet name="Outcomes" sheetId="4" r:id="rId4"/>
+    <sheet name="Assessments" sheetId="5" r:id="rId5"/>
+    <sheet name="Risks" sheetId="6" r:id="rId6"/>
+    <sheet name="Classes" sheetId="7" r:id="rId7"/>
+    <sheet name="GPA" sheetId="8" r:id="rId8"/>
+    <sheet name="Co-curricular" sheetId="9" r:id="rId9"/>
+    <sheet name="Learning Plan" sheetId="10" r:id="rId10"/>
+    <sheet name="Absences" sheetId="11" r:id="rId11"/>
+    <sheet name="Behaviours" sheetId="12" r:id="rId12"/>
+    <sheet name="Health Records" sheetId="13" r:id="rId13"/>
+    <sheet name="Counsellings" sheetId="14" r:id="rId14"/>
+    <sheet name="Cases" sheetId="15" r:id="rId15"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId18" roundtripDataChecksum="9iNyVI1scF3ksjahR7MMfFFn2YeH8aQqbRfGz+eyOZE="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId19" roundtripDataChecksum="QT+J1WNuzP9EuRWRPiy/DbL7D+pcn7GA+ax2ve9/67Y="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="197">
   <si>
     <t>${Institutions.name}/${Institutions.code}</t>
   </si>
@@ -249,6 +250,21 @@
     <t>${"repeatRows":{"displayValue":"CompetencyTemplates.name","children":{"repeatRows":{"displayValue":"CompetencyPeriods.name","filter":"competency_template_id","children":{"repeatRows":{"displayValue":"CompetencyItems.name","filter":"competency_period_id"}}}}}}</t>
   </si>
   <si>
+    <t>Outcome Subject Comments</t>
+  </si>
+  <si>
+    <t>Subject</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>${"repeatRows":{"displayValue":"OutcomeTemplates.name","children":{"repeatRows":{"displayValue":"OutcomePeriods.name","filter":"outcome_template_id","children":{"repeatRows":{"displayValue":"OutcomeSubjects.name","filter":"outcome_period_id"}}}}}}</t>
+  </si>
+  <si>
+    <t>${"match":{"displayValue":"StudentOutcomeSubjectComments.comments","rows":{"matchFrom":"OutcomeTemplates.id","matchTo":"StudentOutcomeSubjectComments.outcome_template_id","children":{"rows":{"matchFrom":"OutcomePeriods.id","matchTo":"StudentOutcomeSubjectComments.outcome_period_id","filter":"outcome_template_id","children":{"rows":{"matchFrom":"OutcomeSubjects.education_subject_id","matchTo":"StudentOutcomeSubjectComments.education_subject_id","filter":"outcome_period_id"}}}}}}}</t>
+  </si>
+  <si>
     <t>Assessments</t>
   </si>
   <si>
@@ -609,10 +625,10 @@
     <t>${"match": {"displayValue": "InstitutionSubjectStudentsWithName.institution_name","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.id","matchTo": "InstitutionSubjectStudentsWithName.id"}}}</t>
   </si>
   <si>
+    <t>${"match": {"displayValue": "InstitutionSubjectStudentsWithName.student_candidate_number","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.id","matchTo": "InstitutionSubjectStudentsWithName.id"}}}</t>
+  </si>
+  <si>
     <t>${"match": {"displayValue": "InstitutionSubjectStudentsWithName.total_mark","type":"number","format":"2","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.education_subject_id","matchTo": "InstitutionSubjectStudentsWithName.education_subject_id"}}}</t>
-  </si>
-  <si>
-    <t>${"match": {"displayValue": "InstitutionSubjectStudentsWithName.student_candidate_number","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.id","matchTo": "InstitutionSubjectStudentsWithName.id"}}}</t>
   </si>
 </sst>
 </file>
@@ -692,7 +708,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -703,12 +719,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF0077D4"/>
         <bgColor rgb="FF0077D4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -881,7 +891,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -912,12 +922,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -993,7 +1003,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2528,6 +2537,1095 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J1000"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="48.90625" customWidth="1"/>
+    <col min="2" max="3" width="36.08984375" customWidth="1"/>
+    <col min="4" max="4" width="18.08984375" customWidth="1"/>
+    <col min="5" max="5" width="32.36328125" customWidth="1"/>
+    <col min="6" max="6" width="21.08984375" customWidth="1"/>
+    <col min="7" max="7" width="15.36328125" customWidth="1"/>
+    <col min="8" max="8" width="27" customWidth="1"/>
+    <col min="9" max="9" width="13.90625" customWidth="1"/>
+    <col min="10" max="10" width="62.453125" customWidth="1"/>
+    <col min="11" max="26" width="8.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="52" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="53" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="54" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="55" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="56" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="57" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="58" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="59" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="60" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="61" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="65" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="66" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="67" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="68" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="69" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="70" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="71" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="72" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="73" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="74" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="75" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="76" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="77" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="78" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="79" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="80" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="81" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="82" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="83" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="84" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="85" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="86" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="87" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="88" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="89" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="90" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="91" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="92" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="93" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="94" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="95" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="96" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="97" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="98" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="99" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="100" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="101" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="102" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="103" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="104" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="105" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="106" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="107" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="108" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="109" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="110" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="111" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="112" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="113" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="114" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="115" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="116" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="117" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="118" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="119" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="120" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="121" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="122" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="123" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="124" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="125" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="126" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="127" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="128" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="129" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="130" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="131" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="132" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="133" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="134" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="135" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="136" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="137" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="138" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="139" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="140" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="141" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="142" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="143" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="144" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="145" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="146" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="147" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="148" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="149" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="150" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="151" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="152" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="153" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="154" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="155" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="156" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="157" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="158" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="159" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="160" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="161" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="162" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="163" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="164" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="165" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="166" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="167" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="168" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="169" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="170" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="171" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="172" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="173" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="174" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="175" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="176" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="177" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="178" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="179" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="180" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="181" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="182" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="183" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="184" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="185" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="186" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="187" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="188" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="189" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="190" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="191" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="192" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="193" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="194" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="195" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="196" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="197" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="198" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="199" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="200" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="201" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="202" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="203" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="204" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="205" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="206" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="207" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="208" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="209" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="210" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="211" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="212" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="213" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="214" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="215" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="216" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="217" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="218" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="219" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="220" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="221" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="222" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="223" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="224" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="225" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="226" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="227" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="228" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="229" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="230" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="231" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="232" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="233" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="234" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="235" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="236" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="237" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="238" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="239" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="240" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="241" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="242" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="243" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="244" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="245" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="246" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="247" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="248" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="249" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="250" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="251" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="252" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="253" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="254" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="255" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="256" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="257" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="258" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="259" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="260" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="261" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="262" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="263" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="264" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="265" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="266" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="267" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="268" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="269" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="270" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="271" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="272" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="273" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="274" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="275" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="276" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="277" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="278" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="279" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="280" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="281" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="282" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="283" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="284" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="285" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="286" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="287" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="288" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="289" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="290" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="291" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="292" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="293" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="294" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="295" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="296" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="297" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="298" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="299" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="300" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="301" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="302" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="303" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="304" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="305" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="306" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="307" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="308" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="309" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="310" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="311" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="312" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="313" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="314" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="315" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="316" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="317" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="318" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="319" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="320" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="321" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="322" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="323" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="324" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="325" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="326" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="327" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="328" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="329" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="330" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="331" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="332" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="333" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="334" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="335" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="336" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="337" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="338" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="339" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="340" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="341" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="342" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="343" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="344" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="345" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="346" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="347" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="348" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="349" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="350" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="351" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="352" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="353" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="354" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="355" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="356" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="357" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="358" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="359" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="360" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="361" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="362" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="363" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="364" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="365" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="366" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="367" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="368" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="369" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="370" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="371" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="372" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="373" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="374" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="375" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="376" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="377" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="378" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="379" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="380" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="381" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="382" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="383" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="384" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="385" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="386" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="387" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="388" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="389" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="390" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="391" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="392" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="393" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="394" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="395" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="396" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="397" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="398" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="399" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="400" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="401" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="402" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="403" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="404" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="405" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="406" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="407" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="408" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="409" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="410" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="411" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="412" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="413" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="414" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="415" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="416" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="417" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="418" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="419" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="420" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="421" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="422" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="423" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="424" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="425" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="426" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="427" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="428" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="429" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="430" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="431" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="432" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="433" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="434" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="435" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="436" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="437" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="438" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="439" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="440" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="441" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="442" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="443" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="444" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="445" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="446" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="447" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="448" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="449" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="450" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="451" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="452" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="453" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="454" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="455" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="456" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="457" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="458" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="459" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="460" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="461" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="462" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="463" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="464" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="465" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="466" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="467" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="468" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="469" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="470" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="471" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="472" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="473" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="474" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="475" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="476" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="477" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="478" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="479" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="480" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="481" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="482" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="483" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="484" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="485" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="486" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="487" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="488" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="489" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="490" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="491" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="492" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="493" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="494" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="495" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="496" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="497" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="498" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="499" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="500" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="501" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="502" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="503" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="504" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="505" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="506" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="507" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="508" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="509" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="510" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="511" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="512" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="513" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="514" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="515" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="516" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="517" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="518" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="519" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="520" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="521" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="522" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="523" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="524" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="525" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="526" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="527" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="528" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="529" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="530" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="531" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="532" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="533" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="534" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="535" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="536" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="537" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="538" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="539" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="540" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="541" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="542" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="543" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="544" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="545" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="546" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="547" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="548" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="549" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="550" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="551" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="552" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="553" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="554" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="555" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="556" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="557" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="558" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="559" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="560" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="561" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="562" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="563" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="564" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="565" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="566" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="567" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="568" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="569" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="570" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="571" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="572" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="573" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="574" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="575" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="576" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="577" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="578" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="579" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="580" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="581" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="582" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="583" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="584" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="585" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="586" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="587" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="588" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="589" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="590" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="591" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="592" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="593" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="594" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="595" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="596" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="597" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="598" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="599" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="600" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="601" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="602" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="603" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="604" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="605" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="606" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="607" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="608" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="609" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="610" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="611" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="612" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="613" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="614" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="615" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="616" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="617" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="618" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="619" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="620" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="621" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="622" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="623" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="624" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="625" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="626" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="627" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="628" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="629" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="630" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="631" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="632" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="633" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="634" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="635" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="636" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="637" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="638" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="639" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="640" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="641" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="642" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="643" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="644" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="645" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="646" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="647" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="648" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="649" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="650" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="651" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="652" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="653" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="654" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="655" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="656" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="657" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="658" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="659" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="660" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="661" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="662" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="663" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="664" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="665" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="666" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="667" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="668" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="669" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="670" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="671" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="672" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="673" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="674" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="675" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="676" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="677" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="678" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="679" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="680" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="681" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="682" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="683" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="684" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="685" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="686" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="687" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="688" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="689" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="690" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="691" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="692" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="693" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="694" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="695" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="696" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="697" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="698" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="699" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="700" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="701" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="702" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="703" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="704" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="705" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="706" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="707" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="708" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="709" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="710" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="711" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="712" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="713" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="714" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="715" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="716" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="717" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="718" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="719" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="720" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="721" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="722" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="723" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="724" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="725" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="726" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="727" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="728" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="729" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="730" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="731" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="732" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="733" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="734" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="735" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="736" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="737" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="738" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="739" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="740" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="741" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="742" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="743" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="744" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="745" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="746" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="747" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="748" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="749" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="750" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="751" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="752" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="753" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="754" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="755" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="756" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="757" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="758" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="759" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="760" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="761" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="762" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="763" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="764" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="765" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="766" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="767" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="768" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="769" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="770" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="771" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="772" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="773" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="774" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="775" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="776" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="777" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="778" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="779" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="780" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="781" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="782" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="783" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="784" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="785" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="786" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="787" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="788" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="789" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="790" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="791" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="792" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="793" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="794" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="795" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="796" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="797" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="798" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="799" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="800" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="801" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="802" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="803" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="804" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="805" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="806" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="807" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="808" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="809" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="810" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="811" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="812" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="813" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="814" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="815" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="816" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="817" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="818" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="819" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="820" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="821" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="822" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="823" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="824" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="825" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="826" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="827" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="828" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="829" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="830" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="831" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="832" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="833" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="834" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="835" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="836" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="837" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="838" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="839" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="840" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="841" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="842" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="843" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="844" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="845" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="846" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="847" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="848" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="849" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="850" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="851" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="852" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="853" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="854" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="855" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="856" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="857" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="858" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="859" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="860" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="861" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="862" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="863" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="864" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="865" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="866" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="867" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="868" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="869" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="870" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="871" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="872" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="873" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="874" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="875" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="876" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="877" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="878" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="879" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="880" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="881" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="882" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="883" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="884" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="885" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="886" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="887" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="888" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="889" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="890" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="891" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="892" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="893" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="894" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="895" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="896" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="897" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="898" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="899" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="900" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="901" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="902" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="903" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="904" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="905" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="906" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="907" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="908" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="909" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="910" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="911" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="912" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="913" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="914" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="915" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="916" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="917" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="918" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="919" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="920" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="921" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="922" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="923" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="924" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="925" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="926" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="927" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="928" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="929" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="930" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="931" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="932" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="933" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="934" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="935" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="936" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="937" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="938" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="939" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="940" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="941" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="942" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="943" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="944" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="945" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="946" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="947" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="948" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="949" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="950" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="951" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="952" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="953" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="954" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="955" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="956" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="957" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="958" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="959" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="960" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="961" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="962" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="963" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="964" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="965" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="966" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="967" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="968" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="969" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="970" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="971" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="972" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="973" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="974" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="975" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="976" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="977" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="978" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="979" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="980" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="981" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="982" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="983" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="984" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="985" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="986" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="987" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="988" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="989" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="990" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="991" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="992" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="993" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="994" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="995" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="996" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="997" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="998" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="999" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1000" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C1000"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2540,58 +3638,58 @@
   <sheetData>
     <row r="1" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="46" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B1" s="47"/>
     </row>
     <row r="2" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="27" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="B2" s="28" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="27" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="27" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="27" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B5" s="28" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="46" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B7" s="47"/>
     </row>
     <row r="8" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="27" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="B8" s="28" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3600,7 +4698,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3613,7 +4711,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="46" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B1" s="42"/>
       <c r="C1" s="42"/>
@@ -3643,25 +4741,25 @@
     </row>
     <row r="2" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="29" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B2" s="30" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C2" s="30" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="F2" s="30" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="G2" s="30" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="H2" s="9"/>
       <c r="I2" s="9"/>
@@ -3685,25 +4783,25 @@
     </row>
     <row r="3" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="31" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B3" s="32" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="D3" s="32" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="E3" s="32" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="F3" s="32" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="G3" s="32" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="H3" s="9"/>
       <c r="I3" s="9"/>
@@ -10594,7 +11692,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D1000"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -10610,7 +11708,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="50" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B1" s="38"/>
       <c r="C1" s="38"/>
@@ -10618,81 +11716,81 @@
     </row>
     <row r="2" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="48" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="B2" s="42"/>
       <c r="C2" s="49" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="D2" s="42"/>
     </row>
     <row r="3" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="48" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B3" s="42"/>
       <c r="C3" s="49" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="D3" s="42"/>
     </row>
     <row r="4" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="48" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B4" s="42"/>
       <c r="C4" s="49" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D4" s="42"/>
     </row>
     <row r="5" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="48" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="B5" s="42"/>
       <c r="C5" s="49" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="D5" s="42"/>
     </row>
     <row r="6" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="48" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B6" s="42"/>
       <c r="C6" s="49" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D6" s="42"/>
     </row>
     <row r="7" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="8" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="20" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -11709,7 +12807,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E1000"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -11723,7 +12821,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="50" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="B1" s="38"/>
       <c r="C1" s="38"/>
@@ -11731,33 +12829,33 @@
     </row>
     <row r="2" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -12770,7 +13868,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E1000"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -12784,7 +13882,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="50" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B1" s="38"/>
       <c r="C1" s="38"/>
@@ -12792,33 +13890,33 @@
     </row>
     <row r="2" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -13870,10 +14968,10 @@
     </row>
     <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>61</v>
@@ -13882,9 +14980,9 @@
         <v>62</v>
       </c>
       <c r="E2" t="s">
-        <v>191</v>
-      </c>
-      <c r="F2" s="51" t="s">
+        <v>195</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>63</v>
       </c>
       <c r="G2" s="4" t="s">
@@ -13908,14 +15006,14 @@
     <col min="1" max="3" width="31.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="43" t="s">
         <v>65</v>
       </c>
       <c r="B1" s="42"/>
       <c r="C1" s="42"/>
     </row>
-    <row r="2" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>66</v>
       </c>
@@ -13926,7 +15024,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>69</v>
       </c>
@@ -13952,62 +15050,114 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="31.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="16" t="s">
+        <v>74</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor theme="6" tint="0.79998168889431442"/>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
   <dimension ref="A1:E9"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="31.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="44" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B1" s="34"/>
       <c r="C1" s="34"/>
       <c r="D1" s="34"/>
       <c r="E1" s="34"/>
     </row>
-    <row r="2" spans="1:5" ht="13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="45" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B2" s="36"/>
       <c r="C2" s="36"/>
       <c r="D2" s="36"/>
       <c r="E2" s="36"/>
     </row>
-    <row r="3" spans="1:5" ht="13" x14ac:dyDescent="0.3">
-      <c r="A3" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="B3" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>74</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="E3" s="18" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>78</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>79</v>
-      </c>
-      <c r="D4" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="E4" s="19" t="s">
-        <v>190</v>
+        <v>82</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -14054,7 +15204,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B1000"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -14067,24 +15217,24 @@
   <sheetData>
     <row r="1" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="46" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B1" s="47"/>
     </row>
     <row r="2" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="21" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -15097,7 +16247,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H1000"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -15116,7 +16266,7 @@
       <c r="B1" s="23"/>
       <c r="C1" s="23"/>
       <c r="D1" s="23" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E1" s="23"/>
       <c r="F1" s="23"/>
@@ -15127,48 +16277,48 @@
         <v>58</v>
       </c>
       <c r="B2" s="24" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D2" s="24" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="E2" s="24" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F2" s="24" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -16178,7 +17328,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D1000"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -16194,36 +17344,36 @@
       <c r="A1" s="23"/>
       <c r="B1" s="23"/>
       <c r="C1" s="23" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D1" s="23"/>
     </row>
     <row r="2" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="24" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B2" s="24" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="D2" s="24" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -17229,7 +18379,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A1000"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -17242,48 +18392,48 @@
   <sheetData>
     <row r="1" spans="1:1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="26" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="1:1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:1" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="10" spans="1:1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="20" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="1:1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -18280,1093 +19430,4 @@
     <oddFooter>&amp;CPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J1000"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="48.90625" customWidth="1"/>
-    <col min="2" max="3" width="36.08984375" customWidth="1"/>
-    <col min="4" max="4" width="18.08984375" customWidth="1"/>
-    <col min="5" max="5" width="32.36328125" customWidth="1"/>
-    <col min="6" max="6" width="21.08984375" customWidth="1"/>
-    <col min="7" max="7" width="15.36328125" customWidth="1"/>
-    <col min="8" max="8" width="27" customWidth="1"/>
-    <col min="9" max="9" width="13.90625" customWidth="1"/>
-    <col min="10" max="10" width="62.453125" customWidth="1"/>
-    <col min="11" max="26" width="8.7265625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-    </row>
-    <row r="9" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="53" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="55" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="67" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="68" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="69" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="70" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="71" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="72" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="73" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="74" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="75" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="76" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="77" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="78" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="79" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="80" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="81" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="82" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="83" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="84" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="85" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="86" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="87" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="88" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="89" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="90" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="91" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="92" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="93" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="94" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="95" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="96" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="97" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="98" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="99" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="100" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="101" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="102" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="103" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="104" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="105" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="106" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="107" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="108" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="109" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="110" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="111" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="112" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="113" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="114" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="115" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="116" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="117" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="118" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="119" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="120" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="121" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="122" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="123" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="124" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="125" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="126" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="127" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="128" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="129" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="130" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="131" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="132" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="133" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="134" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="135" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="136" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="137" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="138" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="139" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="140" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="141" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="142" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="143" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="144" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="145" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="146" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="147" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="148" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="149" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="150" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="151" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="152" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="153" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="154" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="155" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="156" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="157" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="158" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="159" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="160" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="161" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="162" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="163" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="164" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="165" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="166" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="167" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="168" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="169" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="170" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="171" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="172" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="173" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="174" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="175" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="176" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="177" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="178" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="179" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="180" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="181" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="182" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="183" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="184" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="185" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="186" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="187" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="188" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="189" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="190" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="191" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="192" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="193" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="194" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="195" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="196" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="197" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="198" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="199" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="200" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="201" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="202" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="203" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="204" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="205" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="206" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="207" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="208" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="209" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="210" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="211" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="212" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="213" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="214" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="215" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="216" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="217" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="218" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="219" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="220" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="221" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="222" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="223" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="224" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="225" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="226" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="227" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="228" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="229" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="230" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="231" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="232" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="233" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="234" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="235" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="236" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="237" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="238" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="239" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="240" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="241" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="242" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="243" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="244" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="245" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="246" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="247" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="248" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="249" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="250" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="251" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="252" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="253" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="254" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="255" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="256" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="257" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="258" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="259" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="260" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="261" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="262" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="263" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="264" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="265" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="266" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="267" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="268" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="269" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="270" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="271" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="272" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="273" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="274" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="275" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="276" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="277" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="278" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="279" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="280" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="281" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="282" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="283" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="284" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="285" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="286" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="287" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="288" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="289" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="290" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="291" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="292" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="293" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="294" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="295" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="296" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="297" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="298" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="299" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="300" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="301" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="302" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="303" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="304" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="305" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="306" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="307" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="308" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="309" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="310" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="311" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="312" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="313" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="314" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="315" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="316" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="317" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="318" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="319" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="320" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="321" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="322" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="323" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="324" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="325" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="326" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="327" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="328" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="329" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="330" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="331" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="332" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="333" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="334" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="335" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="336" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="337" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="338" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="339" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="340" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="341" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="342" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="343" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="344" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="345" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="346" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="347" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="348" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="349" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="350" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="351" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="352" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="353" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="354" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="355" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="356" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="357" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="358" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="359" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="360" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="361" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="362" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="363" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="364" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="365" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="366" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="367" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="368" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="369" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="370" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="371" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="372" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="373" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="374" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="375" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="376" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="377" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="378" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="379" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="380" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="381" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="382" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="383" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="384" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="385" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="386" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="387" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="388" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="389" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="390" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="391" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="392" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="393" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="394" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="395" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="396" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="397" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="398" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="399" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="400" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="401" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="402" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="403" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="404" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="405" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="406" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="407" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="408" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="409" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="410" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="411" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="412" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="413" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="414" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="415" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="416" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="417" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="418" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="419" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="420" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="421" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="422" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="423" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="424" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="425" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="426" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="427" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="428" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="429" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="430" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="431" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="432" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="433" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="434" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="435" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="436" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="437" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="438" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="439" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="440" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="441" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="442" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="443" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="444" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="445" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="446" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="447" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="448" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="449" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="450" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="451" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="452" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="453" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="454" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="455" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="456" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="457" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="458" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="459" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="460" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="461" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="462" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="463" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="464" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="465" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="466" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="467" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="468" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="469" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="470" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="471" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="472" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="473" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="474" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="475" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="476" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="477" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="478" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="479" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="480" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="481" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="482" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="483" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="484" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="485" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="486" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="487" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="488" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="489" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="490" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="491" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="492" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="493" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="494" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="495" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="496" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="497" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="498" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="499" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="500" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="501" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="502" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="503" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="504" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="505" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="506" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="507" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="508" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="509" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="510" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="511" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="512" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="513" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="514" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="515" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="516" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="517" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="518" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="519" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="520" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="521" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="522" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="523" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="524" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="525" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="526" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="527" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="528" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="529" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="530" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="531" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="532" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="533" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="534" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="535" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="536" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="537" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="538" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="539" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="540" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="541" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="542" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="543" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="544" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="545" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="546" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="547" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="548" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="549" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="550" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="551" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="552" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="553" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="554" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="555" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="556" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="557" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="558" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="559" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="560" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="561" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="562" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="563" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="564" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="565" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="566" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="567" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="568" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="569" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="570" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="571" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="572" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="573" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="574" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="575" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="576" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="577" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="578" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="579" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="580" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="581" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="582" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="583" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="584" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="585" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="586" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="587" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="588" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="589" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="590" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="591" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="592" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="593" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="594" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="595" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="596" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="597" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="598" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="599" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="600" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="601" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="602" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="603" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="604" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="605" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="606" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="607" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="608" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="609" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="610" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="611" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="612" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="613" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="614" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="615" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="616" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="617" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="618" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="619" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="620" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="621" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="622" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="623" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="624" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="625" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="626" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="627" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="628" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="629" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="630" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="631" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="632" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="633" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="634" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="635" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="636" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="637" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="638" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="639" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="640" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="641" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="642" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="643" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="644" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="645" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="646" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="647" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="648" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="649" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="650" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="651" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="652" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="653" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="654" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="655" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="656" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="657" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="658" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="659" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="660" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="661" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="662" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="663" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="664" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="665" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="666" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="667" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="668" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="669" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="670" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="671" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="672" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="673" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="674" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="675" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="676" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="677" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="678" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="679" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="680" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="681" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="682" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="683" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="684" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="685" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="686" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="687" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="688" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="689" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="690" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="691" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="692" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="693" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="694" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="695" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="696" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="697" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="698" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="699" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="700" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="701" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="702" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="703" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="704" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="705" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="706" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="707" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="708" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="709" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="710" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="711" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="712" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="713" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="714" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="715" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="716" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="717" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="718" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="719" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="720" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="721" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="722" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="723" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="724" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="725" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="726" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="727" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="728" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="729" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="730" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="731" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="732" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="733" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="734" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="735" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="736" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="737" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="738" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="739" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="740" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="741" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="742" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="743" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="744" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="745" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="746" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="747" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="748" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="749" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="750" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="751" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="752" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="753" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="754" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="755" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="756" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="757" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="758" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="759" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="760" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="761" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="762" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="763" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="764" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="765" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="766" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="767" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="768" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="769" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="770" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="771" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="772" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="773" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="774" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="775" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="776" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="777" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="778" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="779" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="780" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="781" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="782" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="783" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="784" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="785" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="786" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="787" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="788" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="789" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="790" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="791" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="792" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="793" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="794" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="795" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="796" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="797" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="798" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="799" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="800" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="801" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="802" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="803" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="804" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="805" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="806" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="807" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="808" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="809" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="810" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="811" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="812" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="813" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="814" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="815" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="816" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="817" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="818" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="819" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="820" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="821" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="822" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="823" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="824" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="825" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="826" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="827" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="828" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="829" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="830" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="831" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="832" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="833" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="834" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="835" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="836" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="837" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="838" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="839" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="840" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="841" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="842" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="843" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="844" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="845" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="846" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="847" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="848" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="849" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="850" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="851" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="852" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="853" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="854" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="855" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="856" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="857" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="858" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="859" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="860" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="861" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="862" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="863" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="864" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="865" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="866" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="867" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="868" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="869" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="870" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="871" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="872" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="873" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="874" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="875" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="876" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="877" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="878" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="879" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="880" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="881" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="882" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="883" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="884" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="885" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="886" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="887" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="888" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="889" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="890" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="891" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="892" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="893" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="894" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="895" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="896" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="897" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="898" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="899" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="900" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="901" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="902" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="903" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="904" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="905" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="906" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="907" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="908" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="909" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="910" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="911" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="912" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="913" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="914" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="915" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="916" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="917" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="918" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="919" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="920" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="921" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="922" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="923" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="924" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="925" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="926" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="927" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="928" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="929" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="930" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="931" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="932" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="933" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="934" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="935" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="936" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="937" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="938" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="939" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="940" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="941" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="942" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="943" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="944" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="945" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="946" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="947" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="948" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="949" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="950" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="951" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="952" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="953" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="954" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="955" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="956" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="957" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="958" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="959" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="960" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="961" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="962" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="963" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="964" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="965" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="966" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="967" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="968" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="969" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="970" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="971" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="972" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="973" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="974" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="975" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="976" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="977" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="978" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="979" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="980" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="981" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="982" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="983" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="984" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="985" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="986" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="987" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="988" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="989" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="990" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="991" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="992" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="993" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="994" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="995" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="996" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="997" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="998" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="999" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="1000" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
-</worksheet>
 </file>
</xml_diff>